<commit_message>
Excell Data Exchange Tool Part 4 (Native formulas compatibility, improved UX)
</commit_message>
<xml_diff>
--- a/Assets/Excell Data Exchange/Export/PlayerTuning.xlsx
+++ b/Assets/Excell Data Exchange/Export/PlayerTuning.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet name="Player Tuning" sheetId="1" state="visible" r:id="R9bac8bea55dd438ca7b98bebb98f481f"/>
-    <x:sheet name="_NashCoreTransfer" sheetId="2" state="veryhidden" r:id="Rc7ae37d77fc44cf29b8b7ede7c801cbd"/>
+    <x:sheet name="Player Tuning" sheetId="1" state="visible" r:id="R2016640c4e6845d58ba6b02f1e003e6e"/>
+    <x:sheet name="_TransferData" sheetId="2" state="veryhidden" r:id="Ra2045f80783e40c3a1a70501c211a3ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="0"/>
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
@@ -30,8 +30,15 @@
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -52,6 +59,12 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFB8BAC2"/>
+        <x:bgColor indexed="64"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9D9D9"/>
         <x:bgColor indexed="64"/>
       </x:patternFill>
     </x:fill>
@@ -111,16 +124,16 @@
     </x:border>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFD0D0D0"/>
+        <x:color rgb="FF808080"/>
       </x:left>
       <x:right style="thin">
-        <x:color rgb="FFD0D0D0"/>
+        <x:color rgb="FF808080"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFD0D0D0"/>
+        <x:color rgb="FF808080"/>
       </x:top>
       <x:bottom style="thin">
-        <x:color rgb="FFD0D0D0"/>
+        <x:color rgb="FF808080"/>
       </x:bottom>
       <x:diagonal/>
     </x:border>
@@ -136,7 +149,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="13">
     <x:xf/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -157,24 +170,28 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" applyFont="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf borderId="2" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" applyFont="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" applyFont="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" applyFont="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" applyFont="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" applyFont="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -288,7 +305,9 @@
       <x:c r="A10" t="str" s="6">
         <x:v>MOVEMENT</x:v>
       </x:c>
-      <x:c r="B10" s="7"/>
+      <x:c r="B10" t="n" s="9">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="C10" s="7"/>
       <x:c r="D10" s="7"/>
     </x:row>
@@ -302,7 +321,7 @@
       <x:c r="A12" t="str" s="6">
         <x:v>Base Speed</x:v>
       </x:c>
-      <x:c r="B12" t="n" s="9">
+      <x:c r="B12" t="n" s="10">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C12" t="str" s="6">
@@ -316,7 +335,7 @@
       <x:c r="A13" t="str" s="6">
         <x:v>Max Speed</x:v>
       </x:c>
-      <x:c r="B13" t="n" s="9">
+      <x:c r="B13" t="n" s="10">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C13" t="str" s="6">
@@ -330,7 +349,7 @@
       <x:c r="A14" t="str" s="6">
         <x:v>Acceleration</x:v>
       </x:c>
-      <x:c r="B14" t="n" s="9">
+      <x:c r="B14" t="n" s="10">
         <x:v>-1</x:v>
       </x:c>
       <x:c r="C14" t="str" s="6">
@@ -344,7 +363,7 @@
       <x:c r="A15" t="str" s="6">
         <x:v>Deceleration</x:v>
       </x:c>
-      <x:c r="B15" t="n" s="9">
+      <x:c r="B15" t="n" s="10">
         <x:v>-1</x:v>
       </x:c>
       <x:c r="C15" t="str" s="6">
@@ -372,7 +391,7 @@
       <x:c r="A18" t="str" s="6">
         <x:v>Directions Mode</x:v>
       </x:c>
-      <x:c r="B18" t="str" s="10">
+      <x:c r="B18" t="str" s="11">
         <x:v>All Directions</x:v>
       </x:c>
       <x:c r="C18" t="str" s="6">
@@ -386,7 +405,7 @@
       <x:c r="A19" t="str" s="6">
         <x:v>Front Cone Enabled</x:v>
       </x:c>
-      <x:c r="B19" t="b" s="11">
+      <x:c r="B19" t="b" s="12">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C19" t="str" s="6">
@@ -457,7 +476,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:AR44"/>
+  <x:dimension ref="A1:AR45"/>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str" s="2">
@@ -598,10 +617,10 @@
         <x:v>Workbook</x:v>
       </x:c>
       <x:c r="B2" t="str" s="2">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C2" t="str" s="2">
-        <x:v>2026-07-13T17:26:30.2503927Z</x:v>
+        <x:v>2026-07-13T20:25:53.2367350Z</x:v>
       </x:c>
       <x:c r="D2" t="str" s="2">
         <x:v>ee448e0cc9af4d58a576081f765d81b0</x:v>
@@ -619,7 +638,7 @@
         <x:v>8de2b9c0c65c4537bfcbeaf8041e50ff</x:v>
       </x:c>
       <x:c r="I2" t="str" s="2">
-        <x:v>cac3ee8e6d83cdde0bd57a741cce5bb9063b0236f619fe1f8d63363eb5f2b6e0</x:v>
+        <x:v>e1d49a57344748f74e8a1d63a91beaca9ff5c41ec3543d23aba060472378f5b7</x:v>
       </x:c>
       <x:c r="J2" s="0"/>
       <x:c r="K2" s="0"/>
@@ -4169,6 +4188,106 @@
         <x:v/>
       </x:c>
     </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str" s="2">
+        <x:v>Cell</x:v>
+      </x:c>
+      <x:c r="B45" s="0"/>
+      <x:c r="C45" s="0"/>
+      <x:c r="D45" s="0"/>
+      <x:c r="E45" s="0"/>
+      <x:c r="F45" s="0"/>
+      <x:c r="G45" s="0"/>
+      <x:c r="H45" s="0"/>
+      <x:c r="I45" s="0"/>
+      <x:c r="J45" t="str" s="2">
+        <x:v>381cb682e86e41f093f0523bbd9764a0</x:v>
+      </x:c>
+      <x:c r="K45" t="str" s="2">
+        <x:v>Player Tuning</x:v>
+      </x:c>
+      <x:c r="L45" t="str" s="2">
+        <x:v>Player Tuning</x:v>
+      </x:c>
+      <x:c r="M45" s="0"/>
+      <x:c r="N45" s="0"/>
+      <x:c r="O45" s="0"/>
+      <x:c r="P45" s="0"/>
+      <x:c r="Q45" s="0"/>
+      <x:c r="R45" s="0"/>
+      <x:c r="S45" s="0"/>
+      <x:c r="T45" s="0"/>
+      <x:c r="U45" s="0"/>
+      <x:c r="V45" t="n" s="2">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="W45" t="n" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="X45" t="str" s="2">
+        <x:v>DataField</x:v>
+      </x:c>
+      <x:c r="Y45" t="str" s="2">
+        <x:v>Export</x:v>
+      </x:c>
+      <x:c r="Z45" t="str" s="2">
+        <x:v>Player:aa65d236feea8ab4c8c34e2d8c4b50f3:PlayerControllerPreset:lookSettings.m_DiscreteDirectionMaxSpeedMultipliers.Array.data[0]</x:v>
+      </x:c>
+      <x:c r="AA45" t="str" s="2">
+        <x:v>Player</x:v>
+      </x:c>
+      <x:c r="AB45" t="str" s="2">
+        <x:v>aa65d236feea8ab4c8c34e2d8c4b50f3</x:v>
+      </x:c>
+      <x:c r="AC45" t="str" s="2">
+        <x:v>PlayerControllerPreset</x:v>
+      </x:c>
+      <x:c r="AD45" t="str" s="2">
+        <x:v>Assets/Scriptable Objects/Player/Presets/ConeVision_ForwardAndBarckward.asset</x:v>
+      </x:c>
+      <x:c r="AE45" t="str" s="2">
+        <x:v>Assets/Scriptable Objects/Player/Presets/ConeVision_ForwardAndBarckward.asset</x:v>
+      </x:c>
+      <x:c r="AF45" t="str" s="2">
+        <x:v>lookSettings.m_DiscreteDirectionMaxSpeedMultipliers.Array.data[0]</x:v>
+      </x:c>
+      <x:c r="AG45" t="str" s="2">
+        <x:v>lookSettings.m_DiscreteDirectionMaxSpeedMultipliers.Array.data[]</x:v>
+      </x:c>
+      <x:c r="AH45" t="str" s="2">
+        <x:v>Number</x:v>
+      </x:c>
+      <x:c r="AI45" t="str" s="2">
+        <x:v>Any Field</x:v>
+      </x:c>
+      <x:c r="AJ45" t="str" s="2">
+        <x:v/>
+      </x:c>
+      <x:c r="AK45" t="b" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AL45" t="str" s="2">
+        <x:v/>
+      </x:c>
+      <x:c r="AM45" t="str" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AN45" t="str" s="2">
+        <x:v>0:</x:v>
+      </x:c>
+      <x:c r="AO45" t="str" s="2">
+        <x:v/>
+      </x:c>
+      <x:c r="AP45" t="str" s="2">
+        <x:v/>
+      </x:c>
+      <x:c r="AQ45" t="str" s="2">
+        <x:v/>
+      </x:c>
+      <x:c r="AR45" t="str" s="2">
+        <x:v/>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:drawing r:id="drawing2"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Bugfixing (Style label and boss warnings)
</commit_message>
<xml_diff>
--- a/Assets/Excell Data Exchange/Export/PlayerTuning.xlsx
+++ b/Assets/Excell Data Exchange/Export/PlayerTuning.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet name="Player Tuning" sheetId="1" state="visible" r:id="R2016640c4e6845d58ba6b02f1e003e6e"/>
-    <x:sheet name="_TransferData" sheetId="2" state="veryhidden" r:id="Ra2045f80783e40c3a1a70501c211a3ff"/>
+    <x:sheet name="Player Tuning" sheetId="1" state="visible" r:id="R01369e870c6a4c71b68c9e186e1a9f14"/>
+    <x:sheet name="_TransferData" sheetId="2" state="veryhidden" r:id="Rde9db4066f654a00881d60e092e13d3e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,7 +38,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -59,12 +59,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFB8BAC2"/>
-        <x:bgColor indexed="64"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFD9D9D9"/>
         <x:bgColor indexed="64"/>
       </x:patternFill>
     </x:fill>
@@ -149,7 +143,7 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="12">
     <x:xf/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" textRotation="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -191,10 +185,6 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1" applyFont="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
   </x:cellXfs>
 </x:styleSheet>
 </file>
@@ -305,9 +295,7 @@
       <x:c r="A10" t="str" s="6">
         <x:v>MOVEMENT</x:v>
       </x:c>
-      <x:c r="B10" t="n" s="9">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="B10" s="7"/>
       <x:c r="C10" s="7"/>
       <x:c r="D10" s="7"/>
     </x:row>
@@ -321,7 +309,7 @@
       <x:c r="A12" t="str" s="6">
         <x:v>Base Speed</x:v>
       </x:c>
-      <x:c r="B12" t="n" s="10">
+      <x:c r="B12" t="n" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C12" t="str" s="6">
@@ -335,7 +323,7 @@
       <x:c r="A13" t="str" s="6">
         <x:v>Max Speed</x:v>
       </x:c>
-      <x:c r="B13" t="n" s="10">
+      <x:c r="B13" t="n" s="9">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C13" t="str" s="6">
@@ -349,7 +337,7 @@
       <x:c r="A14" t="str" s="6">
         <x:v>Acceleration</x:v>
       </x:c>
-      <x:c r="B14" t="n" s="10">
+      <x:c r="B14" t="n" s="9">
         <x:v>-1</x:v>
       </x:c>
       <x:c r="C14" t="str" s="6">
@@ -363,7 +351,7 @@
       <x:c r="A15" t="str" s="6">
         <x:v>Deceleration</x:v>
       </x:c>
-      <x:c r="B15" t="n" s="10">
+      <x:c r="B15" t="n" s="9">
         <x:v>-1</x:v>
       </x:c>
       <x:c r="C15" t="str" s="6">
@@ -391,7 +379,7 @@
       <x:c r="A18" t="str" s="6">
         <x:v>Directions Mode</x:v>
       </x:c>
-      <x:c r="B18" t="str" s="11">
+      <x:c r="B18" t="str" s="10">
         <x:v>All Directions</x:v>
       </x:c>
       <x:c r="C18" t="str" s="6">
@@ -405,7 +393,7 @@
       <x:c r="A19" t="str" s="6">
         <x:v>Front Cone Enabled</x:v>
       </x:c>
-      <x:c r="B19" t="b" s="12">
+      <x:c r="B19" t="b" s="11">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C19" t="str" s="6">
@@ -476,7 +464,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:dimension ref="A1:AR45"/>
+  <x:dimension ref="A1:AR44"/>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str" s="2">
@@ -620,7 +608,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C2" t="str" s="2">
-        <x:v>2026-07-13T20:25:53.2367350Z</x:v>
+        <x:v>2026-07-14T07:18:19.7449625Z</x:v>
       </x:c>
       <x:c r="D2" t="str" s="2">
         <x:v>ee448e0cc9af4d58a576081f765d81b0</x:v>
@@ -638,7 +626,7 @@
         <x:v>8de2b9c0c65c4537bfcbeaf8041e50ff</x:v>
       </x:c>
       <x:c r="I2" t="str" s="2">
-        <x:v>e1d49a57344748f74e8a1d63a91beaca9ff5c41ec3543d23aba060472378f5b7</x:v>
+        <x:v>9c1611093716a1877a0e87561502a9ab48179350a6ca01c50a0f01f4489951bc</x:v>
       </x:c>
       <x:c r="J2" s="0"/>
       <x:c r="K2" s="0"/>
@@ -710,7 +698,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="Q3" t="n" s="2">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="R3" t="n" s="2">
         <x:v>1</x:v>
@@ -4188,106 +4176,6 @@
         <x:v/>
       </x:c>
     </x:row>
-    <x:row r="45">
-      <x:c r="A45" t="str" s="2">
-        <x:v>Cell</x:v>
-      </x:c>
-      <x:c r="B45" s="0"/>
-      <x:c r="C45" s="0"/>
-      <x:c r="D45" s="0"/>
-      <x:c r="E45" s="0"/>
-      <x:c r="F45" s="0"/>
-      <x:c r="G45" s="0"/>
-      <x:c r="H45" s="0"/>
-      <x:c r="I45" s="0"/>
-      <x:c r="J45" t="str" s="2">
-        <x:v>381cb682e86e41f093f0523bbd9764a0</x:v>
-      </x:c>
-      <x:c r="K45" t="str" s="2">
-        <x:v>Player Tuning</x:v>
-      </x:c>
-      <x:c r="L45" t="str" s="2">
-        <x:v>Player Tuning</x:v>
-      </x:c>
-      <x:c r="M45" s="0"/>
-      <x:c r="N45" s="0"/>
-      <x:c r="O45" s="0"/>
-      <x:c r="P45" s="0"/>
-      <x:c r="Q45" s="0"/>
-      <x:c r="R45" s="0"/>
-      <x:c r="S45" s="0"/>
-      <x:c r="T45" s="0"/>
-      <x:c r="U45" s="0"/>
-      <x:c r="V45" t="n" s="2">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="W45" t="n" s="2">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="X45" t="str" s="2">
-        <x:v>DataField</x:v>
-      </x:c>
-      <x:c r="Y45" t="str" s="2">
-        <x:v>Export</x:v>
-      </x:c>
-      <x:c r="Z45" t="str" s="2">
-        <x:v>Player:aa65d236feea8ab4c8c34e2d8c4b50f3:PlayerControllerPreset:lookSettings.m_DiscreteDirectionMaxSpeedMultipliers.Array.data[0]</x:v>
-      </x:c>
-      <x:c r="AA45" t="str" s="2">
-        <x:v>Player</x:v>
-      </x:c>
-      <x:c r="AB45" t="str" s="2">
-        <x:v>aa65d236feea8ab4c8c34e2d8c4b50f3</x:v>
-      </x:c>
-      <x:c r="AC45" t="str" s="2">
-        <x:v>PlayerControllerPreset</x:v>
-      </x:c>
-      <x:c r="AD45" t="str" s="2">
-        <x:v>Assets/Scriptable Objects/Player/Presets/ConeVision_ForwardAndBarckward.asset</x:v>
-      </x:c>
-      <x:c r="AE45" t="str" s="2">
-        <x:v>Assets/Scriptable Objects/Player/Presets/ConeVision_ForwardAndBarckward.asset</x:v>
-      </x:c>
-      <x:c r="AF45" t="str" s="2">
-        <x:v>lookSettings.m_DiscreteDirectionMaxSpeedMultipliers.Array.data[0]</x:v>
-      </x:c>
-      <x:c r="AG45" t="str" s="2">
-        <x:v>lookSettings.m_DiscreteDirectionMaxSpeedMultipliers.Array.data[]</x:v>
-      </x:c>
-      <x:c r="AH45" t="str" s="2">
-        <x:v>Number</x:v>
-      </x:c>
-      <x:c r="AI45" t="str" s="2">
-        <x:v>Any Field</x:v>
-      </x:c>
-      <x:c r="AJ45" t="str" s="2">
-        <x:v/>
-      </x:c>
-      <x:c r="AK45" t="b" s="2">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AL45" t="str" s="2">
-        <x:v/>
-      </x:c>
-      <x:c r="AM45" t="str" s="2">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="AN45" t="str" s="2">
-        <x:v>0:</x:v>
-      </x:c>
-      <x:c r="AO45" t="str" s="2">
-        <x:v/>
-      </x:c>
-      <x:c r="AP45" t="str" s="2">
-        <x:v/>
-      </x:c>
-      <x:c r="AQ45" t="str" s="2">
-        <x:v/>
-      </x:c>
-      <x:c r="AR45" t="str" s="2">
-        <x:v/>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:drawing r:id="drawing2"/>
 </x:worksheet>

</xml_diff>